<commit_message>
AFE: alimentación 5 V USB -> TLV75733P, nombres reales (TS922, 1N4148), BoM con adaptadores, conectores de electrodos y micrófono
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V5Cz1Wb6HSRhqzouEW9mso
</commit_message>
<xml_diff>
--- a/docs/afe-emg/BoM_AFE_AuraVox_compacta.xlsx
+++ b/docs/afe-emg/BoM_AFE_AuraVox_compacta.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -544,15 +544,15 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Alcohol isopropilico / gel</t>
+          <t>SOT23 a DIP</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Alcohol isopropilico / gel</t>
+          <t>Adaptador SOT-23-5 a DIP</t>
         </is>
       </c>
       <c r="D5" s="4" t="n"/>
@@ -565,15 +565,15 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>jumper Dupont</t>
+          <t>Alcohol isopropilico / gel</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Cable a Arduino A1..A3 del STM32N6570-DK</t>
+          <t>Alcohol isopropilico / gel</t>
         </is>
       </c>
       <c r="D6" s="4" t="n"/>
@@ -586,15 +586,15 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>broche 4 mm</t>
+          <t>jumper Dupont</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Cable con broche (snap) para electrodo</t>
+          <t>Cable 5 V y GND desde el DK</t>
         </is>
       </c>
       <c r="D7" s="4" t="n"/>
@@ -607,15 +607,15 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>24 AWG rigido</t>
+          <t>jumper Dupont</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Cable para puentes</t>
+          <t>Cable a Arduino A1..A3 del STM32N6570-DK</t>
         </is>
       </c>
       <c r="D8" s="4" t="n"/>
@@ -628,15 +628,15 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>3M Red Dot 2228/2560</t>
+          <t>broche 4 mm a pin</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Electrodo Ag/AgCl con broche</t>
+          <t>Cable de electrodo con broche (snap) 4 mm, idealmente apantallado</t>
         </is>
       </c>
       <c r="D9" s="4" t="n"/>
@@ -649,15 +649,15 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>INA333 modulo MCU-333</t>
+          <t>24 AWG rigido</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>INA333 (modulo MCU-333)</t>
+          <t>Cable para puentes</t>
         </is>
       </c>
       <c r="D10" s="4" t="n"/>
@@ -670,15 +670,15 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>deslizante</t>
+          <t>jumper Dupont</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Interruptor</t>
+          <t>Cables Dupont para el microfono</t>
         </is>
       </c>
       <c r="D11" s="4" t="n"/>
@@ -691,15 +691,15 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>TS922AIYDT</t>
+          <t>header 2.54 mm 1x8 + hembra</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Op-amp doble TS922 (rail-to-rail, 4 MHz)</t>
+          <t>Conector en la placa para los 7 cables</t>
         </is>
       </c>
       <c r="D12" s="4" t="n"/>
@@ -712,15 +712,15 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>10 x 15 cm</t>
+          <t>3M Red Dot 2228/2560</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Perfboard</t>
+          <t>Electrodo Ag/AgCl con broche</t>
         </is>
       </c>
       <c r="D13" s="4" t="n"/>
@@ -733,15 +733,15 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>AA</t>
+          <t>INA333 modulo MCU-333</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Pilas AA</t>
+          <t>INA333 (modulo MCU-333)</t>
         </is>
       </c>
       <c r="D14" s="4" t="n"/>
@@ -754,15 +754,15 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>3xAA</t>
+          <t>INMP441</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Portapilas 3 x AA</t>
+          <t>Modulo microfono digital INMP441 (I2S)</t>
         </is>
       </c>
       <c r="D15" s="4" t="n"/>
@@ -775,15 +775,15 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>MCP1700-3302E TO-92</t>
+          <t>TS922AIYDT</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Regulador LDO 3.3 V</t>
+          <t>Op-amp doble TS922AIYDT (Global 001-TS922)</t>
         </is>
       </c>
       <c r="D16" s="4" t="n"/>
@@ -796,15 +796,15 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2.54 mm</t>
+          <t>10 x 15 cm</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Tira de headers macho/hembra</t>
+          <t>Perfboard</t>
         </is>
       </c>
       <c r="D17" s="4" t="n"/>
@@ -817,15 +817,15 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>DIP-8</t>
+          <t>TLV75733PDBVR</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Zocalo DIP-8</t>
+          <t>Regulador LDO 3.3 V TLV75733PDBVR (Global 014-75733)</t>
         </is>
       </c>
       <c r="D18" s="4" t="n"/>
@@ -838,15 +838,15 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>100p</t>
+          <t>2.54 mm</t>
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>cond. ceramico C0G</t>
+          <t>Tira de headers macho/hembra</t>
         </is>
       </c>
       <c r="D19" s="4" t="n"/>
@@ -859,15 +859,15 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>1n</t>
+          <t>DIP-8</t>
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>cond. ceramico C0G</t>
+          <t>Zocalo DIP-8</t>
         </is>
       </c>
       <c r="D20" s="4" t="n"/>
@@ -880,11 +880,11 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>47p</t>
+          <t>100p</t>
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
@@ -901,15 +901,15 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>100n</t>
+          <t>1n</t>
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>cond. ceramico/electrolitico</t>
+          <t>cond. ceramico C0G</t>
         </is>
       </c>
       <c r="D22" s="4" t="n"/>
@@ -922,15 +922,15 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>10u</t>
+          <t>47p</t>
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>cond. ceramico/electrolitico</t>
+          <t>cond. ceramico C0G</t>
         </is>
       </c>
       <c r="D23" s="4" t="n"/>
@@ -943,11 +943,11 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>1u</t>
+          <t>100n</t>
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
@@ -964,15 +964,15 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>100n</t>
+          <t>10u</t>
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>cond. poliester (film)</t>
+          <t>cond. ceramico/electrolitico</t>
         </is>
       </c>
       <c r="D25" s="4" t="n"/>
@@ -985,15 +985,15 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>15n</t>
+          <t>1u</t>
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>cond. poliester o C0G</t>
+          <t>cond. ceramico/electrolitico</t>
         </is>
       </c>
       <c r="D26" s="4" t="n"/>
@@ -1006,15 +1006,15 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>2.2n</t>
+          <t>100n</t>
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>cond. poliester o C0G</t>
+          <t>cond. poliester (film)</t>
         </is>
       </c>
       <c r="D27" s="4" t="n"/>
@@ -1027,7 +1027,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>68n</t>
+          <t>15n</t>
         </is>
       </c>
       <c r="B28" s="3" t="n">
@@ -1048,15 +1048,15 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>1N4148</t>
+          <t>2.2n</t>
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>diodo</t>
+          <t>cond. poliester o C0G</t>
         </is>
       </c>
       <c r="D29" s="4" t="n"/>
@@ -1069,7 +1069,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>68n</t>
         </is>
       </c>
       <c r="B30" s="3" t="n">
@@ -1077,7 +1077,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>resistencia</t>
+          <t>cond. poliester o C0G</t>
         </is>
       </c>
       <c r="D30" s="4" t="n"/>
@@ -1090,15 +1090,15 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>1N4148</t>
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>resistencia</t>
+          <t>diodo</t>
         </is>
       </c>
       <c r="D31" s="4" t="n"/>
@@ -1111,11 +1111,11 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>10M</t>
+          <t>100</t>
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
@@ -1132,11 +1132,11 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>110k</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="B33" s="3" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
@@ -1153,11 +1153,11 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>1k</t>
+          <t>10M</t>
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
@@ -1174,11 +1174,11 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>2.7k</t>
+          <t>110k</t>
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
@@ -1195,11 +1195,11 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>20k</t>
+          <t>1k</t>
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
@@ -1216,11 +1216,11 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>390k</t>
+          <t>2.7k</t>
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
@@ -1237,7 +1237,7 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>3k</t>
+          <t>20k</t>
         </is>
       </c>
       <c r="B38" s="3" t="n">
@@ -1258,11 +1258,11 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>56k</t>
+          <t>390k</t>
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
@@ -1279,7 +1279,7 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>620k</t>
+          <t>3k</t>
         </is>
       </c>
       <c r="B40" s="3" t="n">
@@ -1300,11 +1300,11 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>75k</t>
+          <t>56k</t>
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
@@ -1319,13 +1319,55 @@
       <c r="F41" s="6" t="n"/>
     </row>
     <row r="42">
-      <c r="D42" s="7" t="inlineStr">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>620k</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>resistencia</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="n"/>
+      <c r="E42" s="5">
+        <f>IF(D42="","",B42*D42)</f>
+        <v/>
+      </c>
+      <c r="F42" s="6" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>75k</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>resistencia</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="n"/>
+      <c r="E43" s="5">
+        <f>IF(D43="","",B43*D43)</f>
+        <v/>
+      </c>
+      <c r="F43" s="6" t="n"/>
+    </row>
+    <row r="44">
+      <c r="D44" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E42" s="8">
-        <f>SUM(E4:E41)</f>
+      <c r="E44" s="8">
+        <f>SUM(E4:E43)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
AFE: ganancia x2500 (MFB x125), Cm0 de bloqueo DC, RLD siempre conectado, estimulo RLC
- MFB: RM1 2.4k, RM2 300k, RM3 2.2k, CM1 150n, CM2 1n (f0 506 Hz, Q 0.545) + Cm0 10u
- RLD: integrador -> RLIM 390k -> electrodo; sin .step ni modos (sin RLD = borrar el cable)
- pasabanda del estimulo sEMG como RLC serie en vez de Laplace
- medidas: VCC, VREF, DC y pico de cada ADC, rafaga/reposo solo AC
- BoM y README actualizados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V5Cz1Wb6HSRhqzouEW9mso
</commit_message>
<xml_diff>
--- a/docs/afe-emg/BoM_AFE_AuraVox_compacta.xlsx
+++ b/docs/afe-emg/BoM_AFE_AuraVox_compacta.xlsx
@@ -968,7 +968,7 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
@@ -1027,7 +1027,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>15n</t>
+          <t>150n</t>
         </is>
       </c>
       <c r="B28" s="3" t="n">
@@ -1048,7 +1048,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>2.2n</t>
+          <t>15n</t>
         </is>
       </c>
       <c r="B29" s="3" t="n">
@@ -1069,7 +1069,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>68n</t>
+          <t>2.2n</t>
         </is>
       </c>
       <c r="B30" s="3" t="n">
@@ -1216,11 +1216,11 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>2.7k</t>
+          <t>2.2k</t>
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
@@ -1237,7 +1237,7 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>20k</t>
+          <t>2.4k</t>
         </is>
       </c>
       <c r="B38" s="3" t="n">
@@ -1258,11 +1258,11 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>390k</t>
+          <t>2.7k</t>
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
@@ -1279,7 +1279,7 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>3k</t>
+          <t>300k</t>
         </is>
       </c>
       <c r="B40" s="3" t="n">
@@ -1300,11 +1300,11 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>56k</t>
+          <t>390k</t>
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
@@ -1321,11 +1321,11 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>620k</t>
+          <t>56k</t>
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
@@ -1342,7 +1342,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>75k</t>
+          <t>620k</t>
         </is>
       </c>
       <c r="B43" s="3" t="n">

</xml_diff>